<commit_message>
Increase size of Comparison of APSIM against Ausfarm
</commit_message>
<xml_diff>
--- a/Tests/Validation/Stock/SheepGrazplanObserved.xlsx
+++ b/Tests/Validation/Stock/SheepGrazplanObserved.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Repos\ApsimX\Tests\Validation\Stock\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7769BFC-7BA9-4AF0-9715-9E395C1C5C5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3B91D30-3F04-4038-ABC1-D8B587736002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="19">
   <si>
     <t>SimulationName</t>
   </si>
@@ -76,16 +76,34 @@
     <t>Amount</t>
   </si>
   <si>
-    <t>Stock.CFleectGrowthAll</t>
+    <t>Stock.IntakeAll.Weight</t>
   </si>
   <si>
-    <t>Stock.IntakeAll.Weight</t>
+    <t>FleeceGrowthRate</t>
+  </si>
+  <si>
+    <t>Stock.IntakeAll.N</t>
+  </si>
+  <si>
+    <t>Stock.RetainedNAll</t>
+  </si>
+  <si>
+    <t>Stock.FaecesAll.N</t>
+  </si>
+  <si>
+    <t>Stock.UrineNAll</t>
+  </si>
+  <si>
+    <t>Stock.MEIntakeAll</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -131,7 +149,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -141,6 +159,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -424,20 +446,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H189"/>
+  <dimension ref="A1:J189"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="31.81640625" customWidth="1"/>
     <col min="2" max="2" width="10.1796875" customWidth="1"/>
-    <col min="3" max="3" width="10.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.6328125" style="1" customWidth="1"/>
     <col min="4" max="4" width="10.81640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.7265625" customWidth="1"/>
     <col min="13" max="13" width="14.453125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="13.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -448,13 +473,28 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" t="s">
         <v>13</v>
       </c>
-      <c r="E1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="F1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="str">
         <f>"Ewes45kgAmount"&amp;B2</f>
         <v>Ewes45kgAmount0</v>
@@ -462,18 +502,32 @@
       <c r="B2" s="2">
         <v>0</v>
       </c>
-      <c r="C2" s="1">
-        <v>-0.27</v>
-      </c>
-      <c r="D2">
+      <c r="C2" s="5">
+        <v>-0.23380000000000001</v>
+      </c>
+      <c r="D2" s="5">
         <v>0</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="6">
+        <v>1.5339999999999999E-2</v>
+      </c>
+      <c r="F2" s="2">
         <v>0</v>
       </c>
-      <c r="F2" s="2"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G2" s="2">
+        <v>-1.8E-3</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>1.8E-3</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="str">
         <f t="shared" ref="A3:A7" si="0">"Ewes45kgAmount"&amp;B3</f>
         <v>Ewes45kgAmount400</v>
@@ -481,18 +535,32 @@
       <c r="B3" s="2">
         <v>400</v>
       </c>
-      <c r="C3" s="1">
-        <v>-6.9000000000000006E-2</v>
-      </c>
-      <c r="D3" s="1">
+      <c r="C3" s="5">
+        <v>-4.1300000000000003E-2</v>
+      </c>
+      <c r="D3" s="5">
         <v>0.4</v>
       </c>
-      <c r="E3" s="2">
-        <v>4.5999999999999996</v>
-      </c>
-      <c r="F3" s="2"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E3" s="6">
+        <v>1.558E-2</v>
+      </c>
+      <c r="F3">
+        <v>1.082E-2</v>
+      </c>
+      <c r="G3">
+        <v>6.9999999999999999E-4</v>
+      </c>
+      <c r="H3">
+        <v>3.2000000000000002E-3</v>
+      </c>
+      <c r="I3">
+        <v>6.8999999999999999E-3</v>
+      </c>
+      <c r="J3">
+        <v>4.9320000000000004</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="str">
         <f t="shared" si="0"/>
         <v>Ewes45kgAmount800</v>
@@ -500,18 +568,32 @@
       <c r="B4" s="2">
         <v>800</v>
       </c>
-      <c r="C4" s="1">
-        <v>6.5000000000000002E-2</v>
-      </c>
-      <c r="D4" s="1">
+      <c r="C4" s="5">
+        <v>8.0199999999999994E-2</v>
+      </c>
+      <c r="D4" s="5">
         <v>0.8</v>
       </c>
-      <c r="E4" s="2">
-        <v>9</v>
-      </c>
-      <c r="F4" s="2"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E4" s="6">
+        <v>1.5820000000000001E-2</v>
+      </c>
+      <c r="F4">
+        <v>2.163E-2</v>
+      </c>
+      <c r="G4">
+        <v>2.1800000000000001E-3</v>
+      </c>
+      <c r="H4">
+        <v>6.7400000000000003E-3</v>
+      </c>
+      <c r="I4">
+        <v>1.2710000000000001E-2</v>
+      </c>
+      <c r="J4">
+        <v>9.86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="str">
         <f t="shared" si="0"/>
         <v>Ewes45kgAmount1200</v>
@@ -519,18 +601,32 @@
       <c r="B5" s="2">
         <v>1200</v>
       </c>
-      <c r="C5" s="1">
-        <v>0.157</v>
-      </c>
-      <c r="D5" s="1">
+      <c r="C5" s="5">
+        <v>0.1804</v>
+      </c>
+      <c r="D5" s="5">
         <v>1.2</v>
       </c>
-      <c r="E5" s="2">
-        <v>15</v>
-      </c>
-      <c r="F5" s="2"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E5" s="6">
+        <v>1.6150000000000001E-2</v>
+      </c>
+      <c r="F5" s="2">
+        <v>3.245E-2</v>
+      </c>
+      <c r="G5">
+        <v>3.3899999999999998E-3</v>
+      </c>
+      <c r="H5">
+        <v>1.051E-2</v>
+      </c>
+      <c r="I5">
+        <v>1.8550000000000001E-2</v>
+      </c>
+      <c r="J5">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="str">
         <f t="shared" si="0"/>
         <v>Ewes45kgAmount1600</v>
@@ -538,18 +634,32 @@
       <c r="B6" s="2">
         <v>1600</v>
       </c>
-      <c r="C6" s="1">
-        <v>0.159</v>
-      </c>
-      <c r="D6" s="1">
-        <v>1.21</v>
-      </c>
-      <c r="E6" s="2">
-        <v>15.2</v>
-      </c>
-      <c r="F6" s="3"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C6" s="5">
+        <v>0.18640000000000001</v>
+      </c>
+      <c r="D6" s="5">
+        <v>1.2239800000000001</v>
+      </c>
+      <c r="E6" s="6">
+        <v>1.617E-2</v>
+      </c>
+      <c r="F6" s="2">
+        <v>3.3099999999999997E-2</v>
+      </c>
+      <c r="G6">
+        <v>3.46E-3</v>
+      </c>
+      <c r="H6">
+        <v>1.074E-2</v>
+      </c>
+      <c r="I6">
+        <v>1.89E-2</v>
+      </c>
+      <c r="J6">
+        <v>15.1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="str">
         <f t="shared" si="0"/>
         <v>Ewes45kgAmount2000</v>
@@ -557,138 +667,380 @@
       <c r="B7" s="4">
         <v>2000</v>
       </c>
-      <c r="C7" s="1">
-        <v>0.159</v>
-      </c>
-      <c r="D7" s="1">
-        <v>1.21</v>
-      </c>
-      <c r="E7" s="2">
-        <v>15.2</v>
-      </c>
-      <c r="F7" s="2"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="3"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-    </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-    </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="C7" s="5">
+        <v>0.18640000000000001</v>
+      </c>
+      <c r="D7" s="5">
+        <v>1.2239800000000001</v>
+      </c>
+      <c r="E7" s="6">
+        <v>1.617E-2</v>
+      </c>
+      <c r="F7" s="2">
+        <v>3.3099999999999997E-2</v>
+      </c>
+      <c r="G7">
+        <v>3.46E-3</v>
+      </c>
+      <c r="H7">
+        <v>1.074E-2</v>
+      </c>
+      <c r="I7">
+        <v>1.89E-2</v>
+      </c>
+      <c r="J7">
+        <v>15.1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" t="str">
+        <f>"Lambs25kgAmount"&amp;B8</f>
+        <v>Lambs25kgAmount0</v>
+      </c>
+      <c r="B8" s="2">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5">
+        <v>-0.21690000000000001</v>
+      </c>
+      <c r="D8" s="5">
+        <v>0</v>
+      </c>
+      <c r="E8" s="6">
+        <v>1.55E-2</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" t="str">
+        <f t="shared" ref="A9:A13" si="1">"Lambs25kgAmount"&amp;B9</f>
+        <v>Lambs25kgAmount400</v>
+      </c>
+      <c r="B9" s="2">
+        <v>400</v>
+      </c>
+      <c r="C9" s="5">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="D9" s="5">
+        <v>0.4</v>
+      </c>
+      <c r="E9" s="6">
+        <v>1.5720000000000001E-2</v>
+      </c>
+      <c r="F9" s="2">
+        <v>1.082E-2</v>
+      </c>
+      <c r="J9">
+        <v>4.9320000000000004</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" t="str">
+        <f t="shared" si="1"/>
+        <v>Lambs25kgAmount800</v>
+      </c>
+      <c r="B10" s="2">
+        <v>800</v>
+      </c>
+      <c r="C10" s="5">
+        <v>0.1615</v>
+      </c>
+      <c r="D10" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="E10" s="6">
+        <v>1.6039999999999999E-2</v>
+      </c>
+      <c r="F10" s="2">
+        <v>2.163E-2</v>
+      </c>
+      <c r="J10">
+        <v>9.8640000000000008</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" t="str">
+        <f t="shared" si="1"/>
+        <v>Lambs25kgAmount1200</v>
+      </c>
+      <c r="B11" s="2">
+        <v>1200</v>
+      </c>
+      <c r="C11" s="5">
+        <v>0.24099999999999999</v>
+      </c>
+      <c r="D11" s="5">
+        <v>1.0476399999999999</v>
+      </c>
+      <c r="E11" s="6">
+        <v>1.626E-2</v>
+      </c>
+      <c r="F11" s="2">
+        <v>2.8330000000000001E-2</v>
+      </c>
+      <c r="J11">
+        <v>12.917</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12" t="str">
+        <f t="shared" si="1"/>
+        <v>Lambs25kgAmount1600</v>
+      </c>
+      <c r="B12" s="2">
+        <v>1600</v>
+      </c>
+      <c r="C12" s="5">
+        <v>0.24099999999999999</v>
+      </c>
+      <c r="D12" s="5">
+        <v>1.0476399999999999</v>
+      </c>
+      <c r="E12" s="6">
+        <v>1.626E-2</v>
+      </c>
+      <c r="F12" s="2">
+        <v>2.8330000000000001E-2</v>
+      </c>
+      <c r="J12">
+        <v>12.917</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" t="str">
+        <f t="shared" si="1"/>
+        <v>Lambs25kgAmount2000</v>
+      </c>
+      <c r="B13" s="4">
+        <v>2000</v>
+      </c>
+      <c r="C13" s="5">
+        <v>0.24099999999999999</v>
+      </c>
+      <c r="D13" s="5">
+        <v>1.0476399999999999</v>
+      </c>
+      <c r="E13" s="6">
+        <v>1.626E-2</v>
+      </c>
+      <c r="F13" s="2">
+        <v>2.8330000000000001E-2</v>
+      </c>
+      <c r="J13">
+        <v>12.917</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A14" t="str">
+        <f>"Ewes45kgLucerneAmount"&amp;B14</f>
+        <v>Ewes45kgLucerneAmount0</v>
+      </c>
+      <c r="B14" s="2">
+        <v>0</v>
+      </c>
+      <c r="C14" s="1">
+        <v>-0.23380000000000001</v>
+      </c>
+      <c r="D14" s="5">
+        <v>0</v>
+      </c>
+      <c r="E14" s="2">
+        <v>1.5339999999999999E-2</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15" t="str">
+        <f t="shared" ref="A15:A19" si="2">"Ewes45kgLucerneAmount"&amp;B15</f>
+        <v>Ewes45kgLucerneAmount400</v>
+      </c>
+      <c r="B15" s="2">
+        <v>400</v>
+      </c>
+      <c r="C15" s="1">
+        <v>-9.4299999999999995E-2</v>
+      </c>
+      <c r="D15" s="5">
+        <v>0.4</v>
+      </c>
+      <c r="E15" s="2">
+        <v>1.5570000000000001E-2</v>
+      </c>
+      <c r="F15" s="2">
+        <v>9.5999999999999992E-3</v>
+      </c>
+      <c r="J15">
+        <v>3.76</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16" t="str">
+        <f t="shared" si="2"/>
+        <v>Ewes45kgLucerneAmount800</v>
+      </c>
+      <c r="B16" s="2">
+        <v>800</v>
+      </c>
+      <c r="C16" s="1">
+        <v>1.77E-2</v>
+      </c>
+      <c r="D16" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="E16" s="2">
+        <v>1.5709999999999998E-2</v>
+      </c>
+      <c r="F16" s="2">
+        <v>1.9199999999999998E-2</v>
+      </c>
+      <c r="J16">
+        <v>7.52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17" t="str">
+        <f t="shared" si="2"/>
+        <v>Ewes45kgLucerneAmount1200</v>
+      </c>
+      <c r="B17" s="2">
+        <v>1200</v>
+      </c>
+      <c r="C17" s="1">
+        <v>5.04E-2</v>
+      </c>
+      <c r="D17" s="5">
+        <v>1.02366</v>
+      </c>
+      <c r="E17" s="2">
+        <v>1.583E-2</v>
+      </c>
+      <c r="F17" s="2">
+        <v>2.4570000000000002E-2</v>
+      </c>
+      <c r="J17">
+        <v>9.6219999999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A18" t="str">
+        <f t="shared" si="2"/>
+        <v>Ewes45kgLucerneAmount1600</v>
+      </c>
+      <c r="B18" s="2">
+        <v>1600</v>
+      </c>
+      <c r="C18" s="1">
+        <v>5.04E-2</v>
+      </c>
+      <c r="D18" s="5">
+        <v>1.02366</v>
+      </c>
+      <c r="E18" s="2">
+        <v>1.583E-2</v>
+      </c>
+      <c r="F18" s="2">
+        <v>2.4570000000000002E-2</v>
+      </c>
+      <c r="J18">
+        <v>9.6219999999999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19" t="str">
+        <f t="shared" si="2"/>
+        <v>Ewes45kgLucerneAmount2000</v>
+      </c>
+      <c r="B19" s="4">
+        <v>2000</v>
+      </c>
+      <c r="C19" s="1">
+        <v>5.04E-2</v>
+      </c>
+      <c r="D19" s="5">
+        <v>1.02366</v>
+      </c>
+      <c r="E19" s="2">
+        <v>1.583E-2</v>
+      </c>
+      <c r="F19" s="2">
+        <v>2.4570000000000002E-2</v>
+      </c>
+      <c r="J19">
+        <v>9.6219999999999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B24" s="2"/>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B25" s="2"/>
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B26" s="2"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B27" s="2"/>
       <c r="E27" s="2"/>
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B28" s="2"/>
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B29" s="2"/>
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B30" s="2"/>
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B31" s="2"/>
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B32" s="2"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>

</xml_diff>